<commit_message>
S9: four new codelists for RISystemBasis; extend columnType and archingModel
New codelists for RISystemBasis's coded fields (diggs-schema S9):
designMethod.xml (4), supportedStructureType.xml (8), safetyFormat.xml (5),
consequenceClass.xml (3, EC7/EN 1990 CC1-CC3 only - ASIRI's domain
classification and EBGEO's load case occupy the same slot but couldn't be
verified from open sources, left for SME confirmation rather than guessed
at).

Extends columnType.xml (S6) and archingModel.xml (S5) with one additional
Occurrence each, pointing at RISystemBasis/riTechniqueType and
RISystemBasis/archingModel respectively, so the program-level statement of
technique family and arching model reuses the same governed vocabulary as
the design- and as-built-level statements rather than forking a second one.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/archingModel.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/archingModel.xlsx
@@ -1704,35 +1704,80 @@
         <f>IF(ISNA(VLOOKUP(B7,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B7" s="2" t="n"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>marston</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>//diggs:RISystemBasis/diggs:archingModel</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8">
         <f>IF(ISNA(VLOOKUP(B8,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B8" s="2" t="n"/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>hewlett_randolph</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>//diggs:RISystemBasis/diggs:archingModel</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9">
         <f>IF(ISNA(VLOOKUP(B9,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B9" s="2" t="n"/>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>zaeske</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>//diggs:RISystemBasis/diggs:archingModel</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10">
         <f>IF(ISNA(VLOOKUP(B10,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B10" s="20" t="n"/>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>adapted_terzaghi</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>//diggs:RISystemBasis/diggs:archingModel</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11">
         <f>IF(ISNA(VLOOKUP(B11,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B11" s="20" t="n"/>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>prandtl</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>//diggs:RISystemBasis/diggs:archingModel</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12">

</xml_diff>